<commit_message>
Auto: Week 30/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W30_2026.xlsx
+++ b/Gulf_Dashboard_W30_2026.xlsx
@@ -474,137 +474,241 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>PRJ-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>LNG Terminal (GMTP)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Noncompliance with EHIA
+The wastewater from the grease trap was being directly discharged into the
+according to discharge
+GMTP-PCC-CAR-037 8 Jul 2026 drainage system on the east side of the temporary site office without In process
+wastewater directly to drainage
+undergoing proper treatment through the wastewater treatment system.
+No segregation of materials and waste was observed, resulting in poor
+Improper waste management
+GMTP-PCC-CAR-038 25 Jul 2026 housekeeping and inadequate waste management practices. In process
+at BOP area
+8.4 SHE NCR Status
+Doc No. Description Issue date Root cause Status
+High-Risk Unsafe Conditions and PCC Tank Civil Subcontractor (CNT) conducted work at height using a 70-
+GMTP-PCC-SHE-NCR-003 Behaviors in Man Basket Lifting 23 Jul 2026 ton crane with a suspended man basket to install anchor bolts on the outer Closed
+Operation wall of the tank at a height exceeding 6 meters.
+Discipline Plan &amp; Actual Approval &amp; Review / Information Construction
+Total This Week Accum. Total This Week Accum.
+Plan 0 29 0 20
+General 35 35 34
+Actual 0 29 0 21</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>- GMTP/PMC/PCC Mass TBT and safety share was cancelled due to Asalha Puja Day. - GMTP/PMC/PCC management TBT and safety award on 5 Aug 2026.
+- SHE/EIA weekly audit was cancelled due to Asalha Puja Day. - SHE/EIA weekly audit on 5 Aug 2026.
+- Big cleaning day on 25 Jul 2026. - Big cleaning day every Saturday.
+- Mentoring program at NongFab school on 24 Jul 2026.
+Security Security
+- Strictly control personnel and vehicle gate pass, check the entrance and exit of materials and - Provided temporary security guard for control personal, vehicle and material at site main gate 24 hours.
+equipment into and out of the projectarea 24/7.(Night shift patrols every 1 hour)
+EIA/EHIA EIA/EHIA
+- Construction site monitoring as EIA/EHIA requirements during 30 Jul – 5 Aug 2026.
+- The Doctor and Nurse give information about health and a basic health check at the CNT
+worker camp on 27 Jul 2026.
+- Concretescraps dumping area audit on 27 Jul 2026.
+Issue for Issue for Document Class
+Approval Construction Z X Y
+General 0 0 0 0 0
+Process 0 0 0 0 0
+Mechanical 0 0 0 0 0
+Mechanical (Tank) 0 0 0 0 0
+Piping 0 0 0 0 0
+Electrical 2 3 1 4 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>PRJ-002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>GOE2-NWT3</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>[PV Farm (GUE)] Expedite skilled worker, scaffolding &amp; tools for install mounting.
+[115kV Transmission Line (PEA, FEC)] Modify drainage along the road of Department of Highway.
+[115kV Transmission Line (PEA, FEC)] Relocate water pipe along the road of Department of Rural Roads</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>PRJ-003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>GSPG-PTN</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>[PV Farm (GUE)] Site Security Issue.
+[PV Farm (GUE)] To expedite electrical work and fulfill the manpower increase commitment
+[PV Farm (GUE)] To expedite civil work for unit sub.
+[PV Farm (GUE)] The rainy season may cause waterlogging across the site.
+[Substation (SIEMENS)] Site Security Issue preventing overtime work on holidays (Friday).
+[Substation (SIEMENS)] To expedite Electrical work.
+[Substation (SIEMENS)] To expedite civil work for the control building.
+[115kV Transmission line (PEA, FEC)] To expedite the delayed foundation work ,concrete pole and top pole installation work.
+[Add Bay (PEA, FEC)] To expedite the delayed civil and Electrical work.
+[Communication / Fiber (PEA, JANUS)] Awaiting 115kV Transmission Line HDD work completion and concrete pole installation to proceed with fiber optic cable pulling. 2</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>PRJ-004</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>GSPG-STN</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>[PV Farm (GUE)] To expedite the secondary electrical work already in progress.
+[Substation (SIEMENS)] To expedite the mobilization of the additional manpower for the Civil works.
+[115 kV Transmission line (PEA, FEC)] Transmission line work in the P84-239 (อบจ.) area has been temporarily suspended due to the pole locations overlapping with the planned future road expansion.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>PRJ-005</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>LNE</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>PRJ-006</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>SSE</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Total Indirect Workforce 58 58 +0
+Total Direct Workforce 108 104 +4</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>PRJ-007</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>SDCE</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>[PV farm (GPD)] GPD issued the Purchase Order to Antai on 24 July 2026. Follow up to ensure the mounting is delivered to site by 28 September 2026, so it does not impact the load rejection test.
+[Transmission Line (PEA&amp;TEC)] Construction permit approval from the Royal Irrigation Department and the Department of Highways is still pending, delaying critical activities (HDD, UG foundations, and MH1/MH2 construction).</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Civil work Civil work
+➢ Steel structure installation at BESS area. ➢ Steel structure installation at BESS area completed.
+➢ Chain-link installation. ➢ Chain-link installation completed.
+Electrical work Electrical work
+➢ Mounting and PV panel installation. ➢ Mounting and PV panel installation.
+➢ DC cable and LV 3C-300 installation completed. ➢ SAT/Individual work completed.
+➢ SAT/Individual work. ➢ MV Cable installation.
+➢ MV Cable installation. ➢ Cable test and IV Curve test.
+➢ Cable test and IV Curve test. ➢ LV cable pulling BESS area.
+➢ LV cable pulling BESS area. ➢ Control cable pulling TR station.
+➢ Control cable pulling TR station. ➢ Fiber optic installation.
+➢ Power received PEA 22kV to SST-03 to BESS Aux panel.
+➢ Chain-link fence and crush rock. ➢ MCC walkdown civil work.
+➢ Power transformer installation completed. ➢ PEA inspect power transformer.
+➢ MV cable for power transformer installation. ➢ Lighting system lux test.
+➢ SCADA system. ➢ Function &amp; interlocking test 115kV, 22kV system.
+➢ MV Cable Hi-pot test. ➢ Fiber optic installation.
+➢ Function &amp; interlocking test 115kV, 22kV system.
+➢ Concrete foundation installation. ➢ Concrete foundation installation.
+➢ Top pole assembly installation. ➢ Top pole assembly installation.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -626,308 +730,824 @@
       <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>PRJ-009</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>AL1 (Alpha 1)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>[Pre-NTP] Along road of route east: observed that certain areas the tree-cutting and houses not yet been cleared.
+[Transmission Line (ENCOM/SCT)] Highway no.41 and steel tower: Kindly expedite approval construction permit for Highway no.41 and conclude the decision steel tower construction, as these matters are significantly impacting the schedule.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>➢ Road excavation at east route.
+➢ Backfill and Compaction at east route
+➢ Continue box culvert construction at route to substation.
+➢ Excavation for WTG03 Foundation.
+➢ Continue TSA access west route.
+➢ Continue rebars cutting, bending for Foundation.
+➢ Rebars installation for WTG06 Foundation.
+➢ Start excavation.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>PRJ-010</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>AL2 (Alpha 2)</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>[CBOP (PCZ)] Requires an additional Soil and Rock Disposal Area with a capacity of approximately 25,600 cubic meters for Central A and Route to WTG.03,06,07
+[TSA (GOLD WIND)] Requires an additional Soil and Rock Disposal Area with a capacity of approximately 99,240 cubic meters for WTG-02,03,04,05,07.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>➢ Continue Cut and Fill for Subgrade layer and Subbase layer Central A, Central B ,Service Road and South
+➢ Continue Pipe and Box culvert South ,Central A ,North A and Service Road
+➢ Continue 33kV Pole Installation
+Actual Completed Deviation
+Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu Fri Sat Sun Mon Tue Wed Thu
+Start Finish
+7/17 7/18 7/19 7/20 7/21 7/22 7/23 7/24 7/25 7/26 7/27 7/28 7/29 7/30 7/31 8/1 8/2 8/3 8/4 8/5 8/6 8/7 8/8 8/9 8/10 8/11 8/12 8/13
+1 North A ( STA.1+400 - STA.4+667 )
+Plan 15-May 16-Aug 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+1 DRAINAGE SYSYTEM ( PIPE &amp; BOX CULVERT )
+Actual 15-May 20.0% -30.0% 0% 0% 0% 0% 0% 0% 0% 2.5% 5% 2.5% 2.5% 0% 5% 2.5%
+Plan 12-Jun 9-Aug 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+2 SLOPE PROTECTION
+Actual 12-Jun 0.0% -50.0% 0% 0% 0% 0% 0% 0% 0% 0% 0% 0% 0% 0% 0% 0%
+Plan 19-Jun 9-Aug 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+3 INSTALLATION ELECTRIC POLE
+Actual 19-Jun 20.0% -30.0% 5% 5% 2.5% 2.5% 2.5% 5% 2.5% 5% 5% 0.0% 2.5% 2.5% 2.5% 2.5%
+2 North B ( STA.0+000 - STA.1+355 )
+Plan 12-Jun 9-Aug 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5% 7.5% 7.5% 7.5% 7.5% 7.5% 7.5% 5%
+1 SLOPE PROTECTION</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>PRJ-011</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>ECE</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>➢ Continue to road base course compaction work.
+➢ Continue to excavation and installation for 33kV Pole.
+➢ Continue to excavation work for drainage system.
+➢ Continue to excavation work.
+➢ Continue to rebar installation.
+➢ Plan to pouring concrete foundation at WTG-07 on 05 August 2026.
+➢ Plan to pouring lean concrete at WTG-05 next week.
+➢ Continue to site preparation (Earth Work).
+➢ Continue to excavation for foundation at SWYD area.
+➢ Start to 115kV foundation rebar installation.
+➢ Continue to foundation work
+➢ Continue to cable Stringing work.
+➢ Continue foundation excavation work.
+➢ Continue to pole installation
+potential hazards and ensure workers understood the work scope.
+activities. ensure compliance.
+Established barricades around the excavation area and installed
+Alcohol level screening for employees entering the project site to Provide PPE according to the risk matrix and regularly inspect its
+warning signage to prevent unauthorized access and ensure site
+prevent work-related hazards and ensure safe operations. proper and safe usage.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>PRJ-012</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>GULF_Wayu</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>[TSA (Goldwind)] The Aor.1 permit approval is currently behind schedule and does not align with the planned start date of the WTG foundation works on 1 June 2026.&gt;&gt;Done
+[CBOP (PCZ)] Bridge and box culvert permit approval is pending. &gt;&gt;Done
+[CBOP (PCZ)] The final COP document has not yet been approved, please expedite the approval process.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>-Plant grass for erosion control.
+-Concrete pole 33kV installation.
+Bridge and Box culvert works
+-Bridge NO.05,06 : Slope protection work.
+-Soil backfill for Box Culvert No. 08.
+-Bridge NO.02A pile driving pier 2,3.
+-RC pipe culvert installation.
+Acc.Plan Last Week Acc.Plan Last Week Acc. Plan
+Acc.Actual Last Week as Plan this week Plan this week Acc. Plan (Contract BL) Acc. Actual this week as
+(Contract BL) (Execution Plan) Delay/Ahead Progress this week (Execution Plan) Delay/Ahead
+No. Work Task %W.V. of 23 Jul 26 (Contract BL) (Execution Plan) as of 30 Jul 26 of 30 Jul 26
+as of 23 Jul 26 as of 23 Jul 26 [B] - [C] of 30 Jul 26 as of 30 Jul 26 [B] - [C]
+[B] as of 30 Jul 26 as of 30 Jul 26 [A] [B]
+[A] [C] [C]
+1 ENGINEERING WORK 5.00% 91.94% 55.40% 53.18% -2.22% 1.74% 0.12% 0.38% 93.68% 55.52% 53.56% -1.96%
+2 PROCUREMENT WORK 55.00% 44.85% 35.40% 35.40% 0.00% 0.72% 0.00% 0.00% 45.57% 35.40% 35.40% 0.00%
+3 CONSTRUCTION WORK 30.00% 8.17% 3.12% 2.99% -0.12% 0.41% 0.72% 0.04% 8.58% 3.84% 3.03% -0.81%
+4 COMMISSIONING WORK 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall Progress 31.72% 23.18% 23.03% -0.15% 0.61% 0.22% 0.03% 32.32% 23.40% 23.06% -0.34%
+➢ Excavation work for WTG-01, WTG-05.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>PRJ-013</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>GCE</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>A conclusion regarding the execution of the manhole, duct bank, and underground piping work has not yet been reached.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Send letter inform equipment transportation
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 90.50% 57.55% -32.95% 92.15% 58.79% -33.36% 92.82%
+Procurement 40.00% 78.91% 77.90% -1.01% 80.66% 78.55% -2.11% 82.61%
+Construction 40.00% 20.13% 13.01% -7.12% 21.48% 13.74% -7.73% 22.90%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 48.67% 42.12% -6.55% 50.07% 42.75% -7.32% 51.49%
+** The data cut off every Friday of week</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>PRJ-014</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>GSE</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Detail and spec of equipment at riser pole for PEA approval.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Plan% Actual% Diff.% Plan% Actual% Diff.% Acc. Plan%
+Engineering 10% 90.50% 57.93% -32.57% 92.15% 58.99% -33.16% 92.82%
+Procurement 40% 78.91% 77.90% -1.01% 80.66% 78.55% -2.11% 82.61%
+Construction 40% 20.13% 16.27% -3.86% 21.48% 16.74% -4.74% 22.90%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 48.67% 43.46% -5.21% 50.07% 44.01% -6.06% 51.49%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 4, Remaining : 0)
+- Total (Finished : 68, Remaining : 0)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Manpower daily report have started to generating automatically at 7:00
+AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 34 prs. Plan to finish &lt;31 Aug 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower
+• Safety training for newcomer</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>PRJ-015</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>KKE</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>311-314 Refuse Bunker Super structure up to 35.5m elevation 9 May 26 23 Nov 26 Delay Start
+325-326 Tipping hall Foundation up to ground (Include piling work) 1 Feb 26 9 Jul 26 8 Feb 26 On going
+327 Tipping hall Super structure up to 13m elevation 10 Jul 26 19 Oct 26
+330-335 Boiler Island &amp; Auxiliary Equipment Foundation 5 Nov 25 14 Jul 26 8 Jan 26 On going
+346 Steam Turbine Generator &amp; Electrical Construction 18 Feb 26 3 Mar 27 8 Feb 26 On going
+408 Holding Pond and Emergency PondConstruction 23 May 26 20 Nov 26
+14 Boiler Arrival at site 12 Jun 26 12 Jun 26
+11 Incinerator Arrival at site 8 May 26 8 May 26 3 May 26 5 May 26 Completed
+15 Steam turbine Arrival at site 2 Oct 26 2 Oct 26
+62- Producing qualified water (Water Receiving date) 23 Feb 27 8 Mar 27
+Stakeholder Management
+Follow up face recognition system
+Follow up foreigner work permit status
+167 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 11 Nov 2025 10
+23 - 29 July
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>(24th Jul 2026) (31st Jul 2026)
+Activities CC/SC (*)
+Plan % Actual % Diff. % Plan % Actual % Diff. % Acc.Plan %
+Engineering 10% 92.55% 59.06% -33.49% 93.41% 60.11% -33.30% 93.75%
+Procurement 40% 84.78% 79.51% -5.27% 86.23% 80.00% -6.23% 86.23%
+Construction 40% 23.65% 19.59% -4.06% 25.39% 20.56% -4.83% 25.39%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 52.62% 45.55% -7.07% 53.99% 46.23% -7.76% 55.23%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.H to make the plan consistent with the actual work.
+(0.00% or more) (-0.01% to – 4.99%) (-5.00% or more)
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)
+Random test alcohol
+Environment &amp; CoP
+Road cleaning</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>PRJ-016</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>MKP</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Multiple key construction milestones have been delayed Manpower, Welder, Scaffolding and formwork shortage</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>(24 Jul 26) (31 Jul 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 77.23 57.71 -19.52 85.40 58.77 -26.63 88.53
+Procurement 40% 73.82 72.87 -0.95 75.19 73.77 -1.42 76.59
+Construction 40% 12.87 13.75 0.88 14.19 15.42 1.23 15.74
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 42.40 40.42 -1.98 44.29 41.55 -2.74 45.75
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>PRJ-017</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>MPE</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BOP Tasks that have started and those that have not yet started are behind schedule
+A conclusion regarding the execution of the manhole, duct bank, and underground piping work has not yet been reached.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 66.19% 57.54% -8.65% 72.27% 58.53% -13.74% 76.94%
+Procurement 40.00% 59.29% 66.43% 7.14% 61.34% 67.56% 6.23% 63.35%
+Construction 40.00% 7.26% 7.67% 0.41% 7.81% 7.97% 0.17% 8.65%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 33.16% 35.39% 2.16% 34.88% 36.07% 1.18% 36.49%
+**Engineering Delay from O &amp; M Manual, Shop Test Report
+On Schedule A Bit Delay Big Delay</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>PRJ-018</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>PFP</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BOP Tasks that have started and those that have not yet started are behind schedule
+A conclusion regarding the execution of the manhole, duct bank, and underground piping work has not yet been reached.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 77.23% 57.19% -20.05% 85.40% 58.18% -27.23% 88.53%
+Procurement 40.00% 73.82% 72.87% -0.96 % 75.19% 73.77% -1.42% 76.59%
+Construction 40.00% 12.87% 8.22% -4.65% 14.19% 10.53% -3.66% 15.74%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 42.40% 38.15% -4.25% 44.29% 39.53% -4.76% 45.78%
+** Engineering delay from O &amp; M Manual, Shop Test Report , Shop ITP
+** Procurement delay from Manufacturing Boiler structure &amp; equipment and Manufacturing STG foundation anchor bolts, condenser metal sheet</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>PRJ-019</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>PKP</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>• Delay in Incinerator and Slag Extractor Installation Due to Material Delivery by 12 Aug 26
+Stakeholder Management
+95 Safety Weekly Audit issue status by weekly
+Total Issues 20
+Since 25 Jan 2026
+Safety Weekly Audit issue Status Chart 23-29 Jul
+Open Closed
+Before After
+Unsafe Condition Not allow to use that access
+HUASHI: Unsafe access way And install barricade
+Government Agencies
+Total of corrective action request EHS issue 1 issue
+Opened 2 issues
+Closed 1 issues
+Closed Open
+No. Date of Discipline Subject Status
+PKP-001-NCR –C -001 9 Mar 26 Civil Embedded Material for Boiler &amp; FGT Delivered does not meet the greed-upon specification Closed
+PKP-001-RFC – C - 001 15 May 26 Civil Request for Clarification on Pile Rig Collapse during Operation of the Causes and Prevention Method Opened
+PKP–002–NCR– S –001 18 Jun. 26 EHS Failure to Implement COP Guidelines in Maintaining the Cleanliness of IEAT Road Opened</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Jul 2026) Jul 2026)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 76.66% 57.25% -19.41% 85.40% 58.24% -27.16% 88.53%
+Procurement 40% 73.82% 72.87% -0.95% 75.19% 73.77% -1.42% 75.59%
+Construction 40% 12.87% 9.45% -3.42% 14.19% 10.07% -4.12% 15.74%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 42.34% 38.65% -3.69% 44.23% 39.36% -4.87% 45.78%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.c to make the plan consistent with the actual work.
+(0.00%or more) (-0.01% to – 4.99%) (-5.00% or more)
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)
+Random test alcohol
+Environment &amp; CoP</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>PRJ-020</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>PSD</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Stakeholder Management
+114 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Jan 2026 10
+23 - 29 July
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Unsafe Condition
+Already improve
+STECON : Unsuitable access way
+Government Agencies
+Problem : Electric Pole obstruct Entrance
+ต ำแหน่งเสำไฟฟ้ำเดมิ
+N.= 1602494.440
+E.= 671208.496
+Entrance ต ำแหน่งเสำไฟฟ้ำใหม่
+▪ ทำ หนังสอื แจง้ ทำง กนอ &gt;&gt; กนอ ทำ หนังสอื แจง้ ทำง PEA &gt;&gt; PEA นครหลวง รบั เรอื งดำ เนินกำรตอ่
+▪ PEA ดำ เนินกำรเรอื งเอกสำรของและเตรยี มทมี ส ำหรบั ทำ งำน ใชเ้วลำโดยประมำณ 1-2 เดอื น
+▪ รำคำโดยประมำณ 100,000 บำท (รอื ถอนเสำไฟฟ้ำเดมิ และตดิ ตงั เสำไฟฟ้ำใหม่)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Key Lookahead Milestones:
+Bunker Building: Lift 1 (EL. -4.5 to +1.0) scheduled for 4–5 Aug (Lift 1 completed).
+Boiler Island: Pouring concrete slab on ground (Z1-Z6)
+FGT : Pouring concrete for ground beam foundation
+STG &amp; ECB: Pouring concrete Slab EL +0.25
+Boiler &amp; Incinerator: Completion of Boiler Drum Installation.
+BOP : Commence foundation work for BOP
+AREA OF CONCERN :
+Bunker Building , Boiler , FGT civil work : Level 3 Schedule update from CEEC is still pending
+Jul 2026) Jul 2026)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 90.50% 57.80% -32.70% 92.15% 58.79% -33.31% 92.82%
+Procurement 40% 78.91% 77.90% -1.01% 80.66% 78.55% -2.11% 82.61%
+Construction 40% 20.13% 11.60% -8.53% 21.48% 13.34% -8.14% 22.90%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 48.67% 41.58% -7.09% 50.07% 42.63% -7.44% 51.49%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.C to make the plan consistent with the actual work.
+(0.00%or more) (-0.01% to – 4.99%) (-5.00% or more)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>PRJ-021</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>PWW1</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>333 Boiler Foundation - Boiler Island 1 May 26 26 June 26 21 May 26 5 Jul 26 Completed
+334 Clearance for boiler installation- Boiler Island 27 June 26 4 July 26 21 May 26 5 Jul 26 Completed
+Piling Work(Including Pile test)- Flue Gas Treatment
+342 2 May 26 30 May 26 4 May 26 19 May 26 Completed
+Equipment Foundation
+Foundation work - Flue Gas Treatment Equipment
+344 11 June 26 21 Aug 26 21 May 26 31 Jul 26 Completed
+Safety Weekly Audit issue status by weekly
+Total Issues 40
+Since 2 Apr 2026
+0 0 0 0 0 0 1 02
+Safety Weekly Audit issue Status Chart
+Open Closed
+Install grounding rod wire on the crane.
+BEFORE AFTER 26
+Soil for backfill PWW1 and PWW2 – Stecon slowly PO process
+• Affect back energize activity
+Pile production for retaining wall (SRF side) – Stecon slowly PO process
+BOP Drawing still not approve
+Service water tank storages – Waiting OE review</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Safety Talk.
+• Safety induction training.
+• Tools and equipment’s inspection.
+• Management walkdown.
+• Random alcohol test.
+• Random drug test.
+Environment &amp; CoP:
+• Water spray to reduce dust.
+• Wheel washing before entering public road.
+• Road cleaning.
+• Bunker wall
+• Continuous Install wall rebar +5.45 to +6.65 m.
+• Mobilize and install slipform (+5.45 m.)
+• Stecon delay mobilize slipform because PO Process
+Activity wall Qty total Qty complete %Complete
+Wall rebar +5.45 to +6.65 m. 4 side 0.5 side 12.50%
+Slipform installation 12 set 0 Set 0.00%
+• Continuous backfill work for ground beam
+• Start column and ground beam rebar work</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>PRJ-022</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>PWW2</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>86 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Apr 2026 10 26 19
+0 0 0 0 0 0 0 01
+Safety Weekly Audit issue Status Chart
+0 Open Closed
+Improper rest area barricade
+Open Closed
+BEFORE AFTER
+Soil for backfill PWW1 and PWW2 – Stecon slowly PO process
+• Affect back energize activity
+Retaining wall (River side) – Stecon scope of work and submit Quotation to CEEC
+• Affect BOP building construction activity
+BOP Drawing still not approve
+Service water tank storages – Waiting OE review
+Cooling tower – Waiting OE review
+Demin water treatment plant – Waiting OE review
+Fire water pump shelter - Waiting OE review and SEPEC update cal.
+Transformer – No calculation for OE review process (Within 15 Aug 26)
+Raw water treatment plant - No drawing (Within (15 Aug 26)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Safety Talk.
+• Safety induction training.
+• Tools and equipment’s inspection.
+• Management walkdown.
+• Random alcohol test.
+• Random drug test.
+Environment &amp; CoP:
+• Water spray to reduce dust.
+• Wheel washing before entering public road.
+• Road cleaning.
+• Refuse bunker wall
+• Continuous install slipform +1.00 m.
+• Start pouring concrete with slipform
+• Bunker building
+• Start ground beam work
+Activity Qty total Qty complete %Complete
+Bunker pit wall – Waterproof membrane 8 side 8 side 100.00%
+Slipform installation 12 set 12 Set 95.00%
+Wall rebar +1.00 to +2.25 m. 4 side 4 side 100.00%</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>PRJ-023</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>TPP</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Multiple key construction milestones have been delayed Manpower, Welder, Scaffolding and formwork shortage</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>(24 Jul 26) (31Jul 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 90.50 57.34 -33.16 92.15 58.59 -33.56 92.82
+Procurement 40% 78.91 77.90 -1.01 80.66 78.55 -2.11 82.61
+Construction 40% 20.13 14.63 -5.50 21.48 17.09 -4.39 22.90
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 48.67 42.77 -5.90 50.07 44.12 -5.95 51.49
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>PRJ-024</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>TSE</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Detail and spec of equipment at riser pole for PEA approval.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Plan% Actual% Diff.% Plan% Actual% Diff.% Acc. Plan%
+Engineering 10% 92.55% 61.52% -31.03% 93.41% 62.94% -30.47% 93.75%
+Procurement 40% 84.78% 79.51% -5.27% 86.23% 80.00% -6.23% 87.53%
+Construction 40% 23.65% 17.84% -5.81% 25.39% 18.10% -7.29% 27.12%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 52.62% 45.09% -7.53% 53.99% 45.53% -8.46% 55.23%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 4, Remaining : 0)
+- Total (Finished : 93, Remaining : 0)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Able to be facial scan 100% (Manpower daily report havealready
+started to generating automatically at 7:00 AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 34 prs. Plan to finish &lt;31 Aug 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower
+• Safety training for newcomer</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -945,46 +1565,113 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>No. Description Progress Remark
+Contractor submitted the Contractor’s
+The contractor has appointed persons to all positions of key personnel and provided a
+representative proposal for the
+detailed organization chart to the employer before the commencement of LNTP works,
+1 Employer’s review. And key
+and for this purpose sub-clause 6.12 of the general conditions shall apply mutatis
+personnel and organization are also
+submitted for review.
+The EPC contractor has sorted out a total of 38 types of permits required for the
+contract to take effect and 33 have been completed.
+No Issue Detail Action by Target ate Progress Remark
+The modifications have been completed according to
+Baseline Schedule and the comments. Currently, we are discussing with the
+1 Submit Project Master Schedule EPC Immediate
+S-curve. OE document control team on how to upload through
+the CNEX system.
+EPC shall maintain a traceable drawing/report
+register, including final quantities, discipline
+2 Design tracking EPC 21/Jul/2026 It will be submitted before the 28.</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>List of Issues to be Coordinated
+Planned (%) (%)
+Design Works 0.404% 17.14% 0.804% 17.946% 0.404% 18.350% 0.404% 18.754%
+Procurement,
+Production &amp; 0.386% 6.73% 0.773% 7.501% 0.386% 7.887% 0.386% 8.274%
+Preparatory
+705% 37.20% 0.605% 37.80% 0.705% 38.505% 0.705% 39.210%
+614% 22.70% 0.614% 23.31% 0.614% 23.927% 0.614% 24.541%
+Construction
+Water Diversion 0.000% 0.00% 0.000% 0.000% 0.000% 0.000% 0.000% 0.000%
+430% 8.44% 0.430% 8.870% 0.430% 9.299% 0.430% 9.729%
+Phase 1 &amp; 2
+PROGRESS 0.193% 4.84% 0.193% 5.06% 0.193% 5.23% 0.193% 5.45%
+(Cumulative %)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>PRJ-026</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Pak Beng</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Right bank abutment、
+Downstream Approach
+Civil 639 623 4 12 164 155 6 3 803 778 10 15
+Channel、R2 Road 、
+Spoil Disposal
+Material、Concrete、
+Test Mortar、Foundation 207 207 0 0 45 45 0 0 252 252 0 0
+bearing capacity
+Total 846 830 4 12 209 200 6 3 1055 1030 10 15
+（For Closing）
+Carry out a mapping of concrete defects
+It was noted that the walls of the drainage along the already built drainage channel.
+channel have many defects, such as 2. Remove the material applied on the
+honeycombs, surface evenness, surface of concrete.
+NCR_No.10misalignment, concrete leakage, cold 31-May-26 3. Submit the Method Statement to carry out / / / Open
+joints, rough surface, etc. Besides this, the reparations and the materials to be used
+bugholes are presented in almost the for OE acceptance.
+entire concrete surface of the walls 4. Send RFI’s to check the preparation of
+defective areas and corrective works.
+Last Month This Month Total</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>PRJ-027</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>TTT</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>To be later</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>